<commit_message>
feat: adopt new vertical score CSV structure in grading pipeline
</commit_message>
<xml_diff>
--- a/HV_Mau 2_Chi tiet KQRL.xlsx
+++ b/HV_Mau 2_Chi tiet KQRL.xlsx
@@ -1606,13 +1606,13 @@
         <v>19</v>
       </c>
       <c r="P18" s="30" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q18" s="33" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S18" s="33" t="n">
         <v>3</v>
@@ -1830,7 +1830,7 @@
         <v>5</v>
       </c>
       <c r="N20" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O20" s="34" t="n">
         <v>20</v>
@@ -2641,7 +2641,7 @@
         <v>20</v>
       </c>
       <c r="P27" s="30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q27" s="33" t="n">
         <v>0</v>
@@ -3331,7 +3331,7 @@
         <v>20</v>
       </c>
       <c r="P33" s="30" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q33" s="33" t="n">
         <v>1</v>
@@ -3527,31 +3527,31 @@
       </c>
       <c r="E35" s="32" t="inlineStr"/>
       <c r="F35" s="30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G35" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H35" s="33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I35" s="33" t="n">
         <v>0</v>
       </c>
       <c r="J35" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="30" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M35" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N35" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O35" s="34" t="n">
         <v>0</v>
@@ -3563,10 +3563,10 @@
         <v>0</v>
       </c>
       <c r="R35" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S35" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T35" s="33" t="n">
         <v>0</v>
@@ -3575,16 +3575,16 @@
         <v>0</v>
       </c>
       <c r="V35" s="30" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="W35" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X35" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y35" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Z35" s="33" t="n">
         <v>0</v>
@@ -4132,7 +4132,7 @@
         <v>20</v>
       </c>
       <c r="P40" s="30" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q40" s="33" t="n">
         <v>0</v>
@@ -4328,31 +4328,31 @@
       </c>
       <c r="E42" s="32" t="inlineStr"/>
       <c r="F42" s="30" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H42" s="33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I42" s="33" t="n">
         <v>0</v>
       </c>
       <c r="J42" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" s="34" t="n">
         <v>0</v>
       </c>
       <c r="L42" s="30" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M42" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N42" s="33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O42" s="34" t="n">
         <v>0</v>
@@ -4364,10 +4364,10 @@
         <v>0</v>
       </c>
       <c r="R42" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S42" s="33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T42" s="33" t="n">
         <v>0</v>
@@ -4376,16 +4376,16 @@
         <v>0</v>
       </c>
       <c r="V42" s="30" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="W42" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="X42" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y42" s="33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Z42" s="33" t="n">
         <v>0</v>
@@ -4570,7 +4570,7 @@
         <v>1</v>
       </c>
       <c r="J44" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="34" t="n">
         <v>16</v>
@@ -4791,7 +4791,7 @@
         <v>3</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H46" s="33" t="n">
         <v>4</v>
@@ -4933,7 +4933,7 @@
         <v>19</v>
       </c>
       <c r="P47" s="30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q47" s="33" t="n">
         <v>0</v>
@@ -5145,7 +5145,7 @@
         <v>1</v>
       </c>
       <c r="J49" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K49" s="34" t="n">
         <v>16</v>

</xml_diff>

<commit_message>
feat: use master Excel totals for class and advisor columns in Word documents
</commit_message>
<xml_diff>
--- a/HV_Mau 2_Chi tiet KQRL.xlsx
+++ b/HV_Mau 2_Chi tiet KQRL.xlsx
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="U18" s="34" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="V18" s="30" t="n">
         <v>8</v>
@@ -1657,11 +1657,11 @@
         <v>0</v>
       </c>
       <c r="AG18" s="35" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="AH18" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI18" s="36" t="n"/>
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="K20" s="34" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L20" s="30" t="n">
         <v>15</v>
@@ -1833,7 +1833,7 @@
         <v>3</v>
       </c>
       <c r="O20" s="34" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="P20" s="30" t="n">
         <v>0</v>
@@ -1887,11 +1887,11 @@
         <v>0</v>
       </c>
       <c r="AG20" s="35" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="AH20" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI20" s="36" t="n"/>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="34" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V27" s="30" t="n">
         <v>8</v>
@@ -2692,11 +2692,11 @@
         <v>0</v>
       </c>
       <c r="AG27" s="35" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="AH27" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI27" s="36" t="n"/>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="34" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="V33" s="30" t="n">
         <v>8</v>
@@ -3382,11 +3382,11 @@
         <v>0</v>
       </c>
       <c r="AG33" s="35" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="AH33" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI33" s="36" t="n"/>
@@ -3542,7 +3542,7 @@
         <v>1</v>
       </c>
       <c r="K35" s="34" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L35" s="30" t="n">
         <v>15</v>
@@ -3554,7 +3554,7 @@
         <v>2</v>
       </c>
       <c r="O35" s="34" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="P35" s="30" t="n">
         <v>0</v>
@@ -3572,7 +3572,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V35" s="30" t="n">
         <v>8</v>
@@ -3593,7 +3593,7 @@
         <v>0</v>
       </c>
       <c r="AB35" s="34" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AC35" s="30" t="n">
         <v>0</v>
@@ -3608,11 +3608,11 @@
         <v>0</v>
       </c>
       <c r="AG35" s="35" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AH35" s="32" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI35" s="36" t="n"/>
@@ -4032,7 +4032,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V39" s="30" t="n">
         <v>8</v>
@@ -4068,11 +4068,11 @@
         <v>0</v>
       </c>
       <c r="AG39" s="35" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AH39" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI39" s="36" t="n"/>
@@ -4147,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="U40" s="34" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V40" s="30" t="n">
         <v>8</v>
@@ -4183,11 +4183,11 @@
         <v>0</v>
       </c>
       <c r="AG40" s="35" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="AH40" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI40" s="36" t="n"/>
@@ -4343,7 +4343,7 @@
         <v>1</v>
       </c>
       <c r="K42" s="34" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L42" s="30" t="n">
         <v>15</v>
@@ -4355,7 +4355,7 @@
         <v>2</v>
       </c>
       <c r="O42" s="34" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="P42" s="30" t="n">
         <v>0</v>
@@ -4373,7 +4373,7 @@
         <v>0</v>
       </c>
       <c r="U42" s="34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V42" s="30" t="n">
         <v>8</v>
@@ -4394,7 +4394,7 @@
         <v>0</v>
       </c>
       <c r="AB42" s="34" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AC42" s="30" t="n">
         <v>0</v>
@@ -4409,11 +4409,11 @@
         <v>0</v>
       </c>
       <c r="AG42" s="35" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AH42" s="32" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI42" s="36" t="n"/>
@@ -4948,7 +4948,7 @@
         <v>0</v>
       </c>
       <c r="U47" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V47" s="30" t="n">
         <v>8</v>
@@ -4984,11 +4984,11 @@
         <v>0</v>
       </c>
       <c r="AG47" s="35" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AH47" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI47" s="36" t="n"/>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="I56" s="49" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="J56" s="48" t="inlineStr">
         <is>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="K56" s="50" t="n">
-        <v>40.54054054054054</v>
+        <v>64.86486486486487</v>
       </c>
       <c r="L56" s="48" t="inlineStr">
         <is>
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="I57" s="49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J57" s="48" t="inlineStr">
         <is>
@@ -5444,7 +5444,7 @@
         </is>
       </c>
       <c r="K57" s="50" t="n">
-        <v>18.91891891891892</v>
+        <v>0</v>
       </c>
       <c r="L57" s="48" t="inlineStr">
         <is>
@@ -5482,7 +5482,7 @@
         </is>
       </c>
       <c r="I59" s="49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J59" s="48" t="inlineStr">
         <is>
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="K59" s="50" t="n">
-        <v>5.405405405405405</v>
+        <v>0</v>
       </c>
       <c r="L59" s="48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs & build: regenerate all student files and update structure documentation
</commit_message>
<xml_diff>
--- a/HV_Mau 2_Chi tiet KQRL.xlsx
+++ b/HV_Mau 2_Chi tiet KQRL.xlsx
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="U18" s="34" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="V18" s="30" t="n">
         <v>8</v>
@@ -1657,11 +1657,11 @@
         <v>0</v>
       </c>
       <c r="AG18" s="35" t="n">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="AH18" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI18" s="36" t="n"/>
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="K20" s="34" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L20" s="30" t="n">
         <v>15</v>
@@ -1833,7 +1833,7 @@
         <v>3</v>
       </c>
       <c r="O20" s="34" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="P20" s="30" t="n">
         <v>0</v>
@@ -1887,11 +1887,11 @@
         <v>0</v>
       </c>
       <c r="AG20" s="35" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AH20" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI20" s="36" t="n"/>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="34" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="V27" s="30" t="n">
         <v>8</v>
@@ -2692,11 +2692,11 @@
         <v>0</v>
       </c>
       <c r="AG27" s="35" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AH27" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI27" s="36" t="n"/>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="34" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V33" s="30" t="n">
         <v>8</v>
@@ -3382,11 +3382,11 @@
         <v>0</v>
       </c>
       <c r="AG33" s="35" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="AH33" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI33" s="36" t="n"/>
@@ -3542,7 +3542,7 @@
         <v>1</v>
       </c>
       <c r="K35" s="34" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L35" s="30" t="n">
         <v>15</v>
@@ -3554,7 +3554,7 @@
         <v>2</v>
       </c>
       <c r="O35" s="34" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="P35" s="30" t="n">
         <v>0</v>
@@ -3572,7 +3572,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V35" s="30" t="n">
         <v>8</v>
@@ -3593,7 +3593,7 @@
         <v>0</v>
       </c>
       <c r="AB35" s="34" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="AC35" s="30" t="n">
         <v>0</v>
@@ -3608,11 +3608,11 @@
         <v>0</v>
       </c>
       <c r="AG35" s="35" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="AH35" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Kém</t>
         </is>
       </c>
       <c r="AI35" s="36" t="n"/>
@@ -4032,7 +4032,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="34" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V39" s="30" t="n">
         <v>8</v>
@@ -4068,11 +4068,11 @@
         <v>0</v>
       </c>
       <c r="AG39" s="35" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="AH39" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI39" s="36" t="n"/>
@@ -4147,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="U40" s="34" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V40" s="30" t="n">
         <v>8</v>
@@ -4183,11 +4183,11 @@
         <v>0</v>
       </c>
       <c r="AG40" s="35" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="AH40" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI40" s="36" t="n"/>
@@ -4343,7 +4343,7 @@
         <v>1</v>
       </c>
       <c r="K42" s="34" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L42" s="30" t="n">
         <v>15</v>
@@ -4355,7 +4355,7 @@
         <v>2</v>
       </c>
       <c r="O42" s="34" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="P42" s="30" t="n">
         <v>0</v>
@@ -4373,7 +4373,7 @@
         <v>0</v>
       </c>
       <c r="U42" s="34" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V42" s="30" t="n">
         <v>8</v>
@@ -4394,7 +4394,7 @@
         <v>0</v>
       </c>
       <c r="AB42" s="34" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="AC42" s="30" t="n">
         <v>0</v>
@@ -4409,11 +4409,11 @@
         <v>0</v>
       </c>
       <c r="AG42" s="35" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="AH42" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Kém</t>
         </is>
       </c>
       <c r="AI42" s="36" t="n"/>
@@ -4948,7 +4948,7 @@
         <v>0</v>
       </c>
       <c r="U47" s="34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V47" s="30" t="n">
         <v>8</v>
@@ -4984,11 +4984,11 @@
         <v>0</v>
       </c>
       <c r="AG47" s="35" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AH47" s="32" t="inlineStr">
         <is>
-          <t>Khá</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="AI47" s="36" t="n"/>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="I56" s="49" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="J56" s="48" t="inlineStr">
         <is>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="K56" s="50" t="n">
-        <v>64.86486486486487</v>
+        <v>40.54054054054054</v>
       </c>
       <c r="L56" s="48" t="inlineStr">
         <is>
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="I57" s="49" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J57" s="48" t="inlineStr">
         <is>
@@ -5444,7 +5444,7 @@
         </is>
       </c>
       <c r="K57" s="50" t="n">
-        <v>0</v>
+        <v>18.91891891891892</v>
       </c>
       <c r="L57" s="48" t="inlineStr">
         <is>
@@ -5482,7 +5482,7 @@
         </is>
       </c>
       <c r="I59" s="49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J59" s="48" t="inlineStr">
         <is>
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="K59" s="50" t="n">
-        <v>0</v>
+        <v>5.405405405405405</v>
       </c>
       <c r="L59" s="48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: document scoring rules, fix student name-splitting logic, resolve mathematical inconsistencies, and correct meeting attendance scores
</commit_message>
<xml_diff>
--- a/HV_Mau 2_Chi tiet KQRL.xlsx
+++ b/HV_Mau 2_Chi tiet KQRL.xlsx
@@ -1482,7 +1482,7 @@
         <v>15</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N17" s="33" t="n">
         <v>0</v>
@@ -1497,7 +1497,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S17" s="33" t="n">
         <v>3</v>
@@ -1585,7 +1585,7 @@
         <v>4</v>
       </c>
       <c r="I18" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="33" t="n">
         <v>1</v>
@@ -1621,19 +1621,19 @@
         <v>0</v>
       </c>
       <c r="U18" s="34" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="V18" s="30" t="n">
         <v>8</v>
       </c>
       <c r="W18" s="33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X18" s="33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Y18" s="33" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Z18" s="33" t="n">
         <v>0</v>
@@ -1657,11 +1657,11 @@
         <v>0</v>
       </c>
       <c r="AG18" s="35" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="AH18" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI18" s="36" t="n"/>
@@ -1712,7 +1712,7 @@
         <v>15</v>
       </c>
       <c r="M19" s="33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N19" s="33" t="n">
         <v>1</v>
@@ -1721,10 +1721,10 @@
         <v>18</v>
       </c>
       <c r="P19" s="30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R19" s="33" t="n">
         <v>1</v>
@@ -1809,7 +1809,7 @@
         <v>3</v>
       </c>
       <c r="G20" s="33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H20" s="33" t="n">
         <v>4</v>
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="K20" s="34" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L20" s="30" t="n">
         <v>15</v>
@@ -1833,7 +1833,7 @@
         <v>3</v>
       </c>
       <c r="O20" s="34" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="P20" s="30" t="n">
         <v>0</v>
@@ -1887,11 +1887,11 @@
         <v>0</v>
       </c>
       <c r="AG20" s="35" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="AH20" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI20" s="36" t="n"/>
@@ -2154,7 +2154,7 @@
         <v>3</v>
       </c>
       <c r="G23" s="33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H23" s="33" t="n">
         <v>4</v>
@@ -2641,10 +2641,10 @@
         <v>20</v>
       </c>
       <c r="P27" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q27" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" s="33" t="n">
         <v>0</v>
@@ -2656,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="34" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V27" s="30" t="n">
         <v>8</v>
@@ -2692,11 +2692,11 @@
         <v>0</v>
       </c>
       <c r="AG27" s="35" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="AH27" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI27" s="36" t="n"/>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
       <c r="U33" s="34" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="V33" s="30" t="n">
         <v>8</v>
@@ -3382,11 +3382,11 @@
         <v>0</v>
       </c>
       <c r="AG33" s="35" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="AH33" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI33" s="36" t="n"/>
@@ -3542,7 +3542,7 @@
         <v>1</v>
       </c>
       <c r="K35" s="34" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L35" s="30" t="n">
         <v>15</v>
@@ -3551,10 +3551,10 @@
         <v>5</v>
       </c>
       <c r="N35" s="33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O35" s="34" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="P35" s="30" t="n">
         <v>0</v>
@@ -3572,13 +3572,13 @@
         <v>0</v>
       </c>
       <c r="U35" s="34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V35" s="30" t="n">
         <v>8</v>
       </c>
       <c r="W35" s="33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X35" s="33" t="n">
         <v>5</v>
@@ -3593,7 +3593,7 @@
         <v>0</v>
       </c>
       <c r="AB35" s="34" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AC35" s="30" t="n">
         <v>0</v>
@@ -3608,11 +3608,11 @@
         <v>0</v>
       </c>
       <c r="AG35" s="35" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AH35" s="32" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI35" s="36" t="n"/>
@@ -4032,7 +4032,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V39" s="30" t="n">
         <v>8</v>
@@ -4068,11 +4068,11 @@
         <v>0</v>
       </c>
       <c r="AG39" s="35" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AH39" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI39" s="36" t="n"/>
@@ -4147,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="U40" s="34" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V40" s="30" t="n">
         <v>8</v>
@@ -4183,11 +4183,11 @@
         <v>0</v>
       </c>
       <c r="AG40" s="35" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="AH40" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI40" s="36" t="n"/>
@@ -4343,7 +4343,7 @@
         <v>1</v>
       </c>
       <c r="K42" s="34" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L42" s="30" t="n">
         <v>15</v>
@@ -4352,10 +4352,10 @@
         <v>5</v>
       </c>
       <c r="N42" s="33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O42" s="34" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="P42" s="30" t="n">
         <v>0</v>
@@ -4373,13 +4373,13 @@
         <v>0</v>
       </c>
       <c r="U42" s="34" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="V42" s="30" t="n">
         <v>8</v>
       </c>
       <c r="W42" s="33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X42" s="33" t="n">
         <v>5</v>
@@ -4394,7 +4394,7 @@
         <v>0</v>
       </c>
       <c r="AB42" s="34" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AC42" s="30" t="n">
         <v>0</v>
@@ -4409,11 +4409,11 @@
         <v>0</v>
       </c>
       <c r="AG42" s="35" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="AH42" s="32" t="inlineStr">
         <is>
-          <t>Kém</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI42" s="36" t="n"/>
@@ -4588,10 +4588,10 @@
         <v>21</v>
       </c>
       <c r="P44" s="30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q44" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R44" s="33" t="n">
         <v>3</v>
@@ -4703,10 +4703,10 @@
         <v>20</v>
       </c>
       <c r="P45" s="30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q45" s="33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R45" s="33" t="n">
         <v>3</v>
@@ -4791,7 +4791,7 @@
         <v>3</v>
       </c>
       <c r="G46" s="33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H46" s="33" t="n">
         <v>4</v>
@@ -4948,7 +4948,7 @@
         <v>0</v>
       </c>
       <c r="U47" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V47" s="30" t="n">
         <v>8</v>
@@ -4984,11 +4984,11 @@
         <v>0</v>
       </c>
       <c r="AG47" s="35" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AH47" s="32" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Khá</t>
         </is>
       </c>
       <c r="AI47" s="36" t="n"/>
@@ -5154,10 +5154,10 @@
         <v>15</v>
       </c>
       <c r="M49" s="33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N49" s="33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O49" s="34" t="n">
         <v>22</v>
@@ -5251,7 +5251,7 @@
         <v>3</v>
       </c>
       <c r="G50" s="41" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H50" s="41" t="n">
         <v>4</v>
@@ -5413,7 +5413,7 @@
         </is>
       </c>
       <c r="I56" s="49" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="J56" s="48" t="inlineStr">
         <is>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="K56" s="50" t="n">
-        <v>40.54054054054054</v>
+        <v>64.86486486486487</v>
       </c>
       <c r="L56" s="48" t="inlineStr">
         <is>
@@ -5436,7 +5436,7 @@
         </is>
       </c>
       <c r="I57" s="49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J57" s="48" t="inlineStr">
         <is>
@@ -5444,7 +5444,7 @@
         </is>
       </c>
       <c r="K57" s="50" t="n">
-        <v>18.91891891891892</v>
+        <v>0</v>
       </c>
       <c r="L57" s="48" t="inlineStr">
         <is>
@@ -5482,7 +5482,7 @@
         </is>
       </c>
       <c r="I59" s="49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J59" s="48" t="inlineStr">
         <is>
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="K59" s="50" t="n">
-        <v>5.405405405405405</v>
+        <v>0</v>
       </c>
       <c r="L59" s="48" t="inlineStr">
         <is>

</xml_diff>